<commit_message>
Update folder.xlsx in deploy directory
</commit_message>
<xml_diff>
--- a/deploy/folder.xlsx
+++ b/deploy/folder.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\xampp\htdocs\spreadsheet-reader\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Program Files\MAMP\htdocs\simlurah_dev\deploy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC070433-B39E-4C63-A0DF-1804B9205462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8892AB15-AEEC-4D96-BB7E-756DFC4D377F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FOLDER SIMLURAH" sheetId="1" r:id="rId1"/>
@@ -33,49 +33,49 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
-    <t>../makassarkec/</t>
-  </si>
-  <si>
-    <t>../biringkanayakec/</t>
-  </si>
-  <si>
-    <t>../bontoalakec/</t>
-  </si>
-  <si>
-    <t>../tamalanreakec/</t>
-  </si>
-  <si>
-    <t>../ujungpandangkec/</t>
-  </si>
-  <si>
-    <t>../tamalatekec/</t>
-  </si>
-  <si>
-    <t>../wajokec/</t>
-  </si>
-  <si>
-    <t>../panakkukangkec/</t>
-  </si>
-  <si>
-    <t>../tallokec/</t>
-  </si>
-  <si>
-    <t>../marisokec/</t>
-  </si>
-  <si>
-    <t>../mamajangkec/</t>
-  </si>
-  <si>
-    <t>../manggalakec/</t>
-  </si>
-  <si>
-    <t>../rappocinikec/</t>
-  </si>
-  <si>
-    <t>../ujungtanahkec/</t>
-  </si>
-  <si>
-    <t>../kepsangkarrangkec/</t>
+    <t>../../makassarkec/</t>
+  </si>
+  <si>
+    <t>../../biringkanayakec/</t>
+  </si>
+  <si>
+    <t>../../bontoalakec/</t>
+  </si>
+  <si>
+    <t>../../tamalanreakec/</t>
+  </si>
+  <si>
+    <t>../../ujungpandangkec/</t>
+  </si>
+  <si>
+    <t>../../tamalatekec/</t>
+  </si>
+  <si>
+    <t>../../wajokec/</t>
+  </si>
+  <si>
+    <t>../../panakkukangkec/</t>
+  </si>
+  <si>
+    <t>../../tallokec/</t>
+  </si>
+  <si>
+    <t>../../marisokec/</t>
+  </si>
+  <si>
+    <t>../../mamajangkec/</t>
+  </si>
+  <si>
+    <t>../../manggalakec/</t>
+  </si>
+  <si>
+    <t>../../rappocinikec/</t>
+  </si>
+  <si>
+    <t>../../ujungtanahkec/</t>
+  </si>
+  <si>
+    <t>../../kepsangkarrangkec/</t>
   </si>
 </sst>
 </file>
@@ -428,82 +428,82 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="82.140625" customWidth="1"/>
+    <col min="1" max="1" width="82.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>14</v>
       </c>

</xml_diff>